<commit_message>
Apply survey areas at WSE 37.28 (543 m2) and 39.5 (1932 m2)
Update the stage-storage guide with the user's delineated inundation areas
and clarify WSE = water surface elevation in the start sheet.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Stage_Storage_Discharge_Guide_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Stage_Storage_Discharge_Guide_900.xlsx
@@ -2034,7 +2034,7 @@
         <v>37.28</v>
       </c>
       <c r="B16" s="14" t="n">
-        <v>600</v>
+        <v>543</v>
       </c>
       <c r="C16" s="10">
         <f>A16-A15</f>
@@ -2084,7 +2084,7 @@
         <v>39.5</v>
       </c>
       <c r="B18" s="14" t="n">
-        <v>1032</v>
+        <v>1932</v>
       </c>
       <c r="C18" s="7">
         <f>A18-A17</f>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Your 1032 m² example — optional higher stage, not the 2.4 link</t>
+          <t>Your 1932 m² example — optional higher stage, not the 2.4 link</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Cell E for the 37.28 m row = total water volume (m³) stored in the landscape when the free surface is at 37.28 m (starting from empty at invert). REPLACE the yellow Area at 37.28 with the area your boss delineated (or that you redraw at 37.28). Placeholder areas above are FAKE except 39.5→1032 which you measured — they only show the method.</t>
+          <t>Cell E for the 37.28 m row = total water volume (m³) stored in the landscape when the free surface is at 37.28 m (starting from empty at invert). REPLACE the yellow Area at 37.28 with the area your boss delineated (or that you redraw at 37.28). Placeholder areas above are FAKE except 39.5→1932 which you measured — they only show the method.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix guide script syntax and regenerate Excel with WSE notes
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Stage_Storage_Discharge_Guide_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Stage_Storage_Discharge_Guide_900.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1286,6 +1286,61 @@
       <c r="A38" t="inlineStr">
         <is>
           <t>Yellow cells = you may edit. Green = results. Orange = boss design stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>WHAT IS WSE?</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>WSE = Water Surface Elevation = the elevation of the free water surface (metres).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Example: WSE = 37.28 m means the water surface is at elevation 37.28 on the survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>YOUR MEASURED AREAS (applied in sheet 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WSE 37.28 m → Area ≈ 543 m²   (boss / +1.5 m above crown stage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WSE 39.50 m → Area ≈ 1932 m²  (optional higher stage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Intermediate WSEs still use placeholder areas until you delineate them.</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2169,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Cell E for the 37.28 m row = total water volume (m³) stored in the landscape when the free surface is at 37.28 m (starting from empty at invert). REPLACE the yellow Area at 37.28 with the area your boss delineated (or that you redraw at 37.28). Placeholder areas above are FAKE except 39.5→1932 which you measured — they only show the method.</t>
+          <t>Cell E for the 37.28 m row = total water volume (m³) stored in the landscape when the free surface is at 37.28 m (starting from empty at invert). REPLACE the yellow Area at 37.28 with the area your boss delineated (or that you redraw at 37.28). Areas at 37.28 m (543 m²) and 39.5 m (1932 m²) are YOUR survey values. Other yellow areas are still placeholders until you delineate those contours.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Translate 4_STAGE_STORAGE sheet to French
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Stage_Storage_Discharge_Guide_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Stage_Storage_Discharge_Guide_900.xlsx
@@ -337,7 +337,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Stage–storage V(WSE)</a:t>
+              <a:t>Cote–stockage V(NSE)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -396,7 +396,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>WSE (m)</a:t>
+                  <a:t>NSE / WSE (m)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1885,25 +1885,25 @@
   <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stage–storage: V = f(WSE) from survey areas</t>
+          <t>Cote–stockage : V = f(NSE) à partir des surfaces topographiques</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>For EACH water level below, draw the inundation polygon on the topo and type the AREA (m²) in yellow. Volume between two levels uses the trapezoid rule in plain text: V_step = (A_i + A_i+1) / 2 * (WSE_i+1 - WSE_i). Cumulative V = sum of steps from the bottom up.</t>
+          <t>NSE = niveau de la surface d'eau (Water Surface Elevation, WSE). Pour CHAQUE niveau d'eau ci-dessous, dessinez le polygone d'inondation sur le topo et inscrivez la SURFACE A (m²) dans les cellules jaunes. Le volume entre deux niveaux utilise la règle des trapèzes : V_pas = (A_i + A_i+1) / 2 × (NSE_i+1 − NSE_i). V cumulatif = somme des V_pas depuis le radier jusqu'au niveau considéré.</t>
         </is>
       </c>
     </row>
@@ -1912,53 +1912,53 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Plain formula for one step</t>
+          <t>Formule en clair pour un pas</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>V_step (m³) = (Area_low + Area_high) / 2  ×  (WSE_high − WSE_low)</t>
+          <t>V_pas (m³) = (Surface_basse + Surface_haute) / 2  ×  (NSE_haute − NSE_basse)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>V_cumulative at a level = sum of all V_step from invert up to that level</t>
+          <t>V_cumulatif à un niveau = somme de tous les V_pas depuis le radier jusqu'à ce niveau</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>WSE (m)</t>
+          <t>NSE / WSE (m)</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Area A (m²)  ← EDIT</t>
+          <t>Surface A (m²)  ← ÉDITER</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>ΔWSE (m)</t>
+          <t>ΔNSE (m)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>V_step (m³)</t>
+          <t>V_pas (m³)</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>V_cumulative (m³)</t>
+          <t>V_cumulatif (m³)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Rôle</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Invert — start (area often 0)</t>
+          <t>Radier — départ (surface souvent 0)</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Intermediate contour — replace with survey area</t>
+          <t>Courbe intermédiaire — remplacer par la surface du levé</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Intermediate contour — replace with survey area</t>
+          <t>Courbe intermédiaire — remplacer par la surface du levé</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Intermediate contour — replace with survey area</t>
+          <t>Courbe intermédiaire — remplacer par la surface du levé</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Intermediate contour — replace with survey area</t>
+          <t>Courbe intermédiaire — remplacer par la surface du levé</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>BOSS LIMIT — replace Area with YOUR delineation at 37.28 m</t>
+          <t>LIMITE PATRON — surface à 37,28 m (votre relevé : 543 m²) ; Qout = 2,4 m³/s</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Intermediate contour — replace with survey area</t>
+          <t>Courbe intermédiaire — remplacer par la surface du levé</t>
         </is>
       </c>
     </row>
@@ -2155,21 +2155,21 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Your 1932 m² example — optional higher stage, not the 2.4 link</t>
+          <t>Votre surface 1932 m² — niveau optionnel plus haut, pas le lien à Q=2,4</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Worked meaning of V at 37.28 m</t>
+          <t>Signification de V à 37,28 m</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Cell E for the 37.28 m row = total water volume (m³) stored in the landscape when the free surface is at 37.28 m (starting from empty at invert). REPLACE the yellow Area at 37.28 with the area your boss delineated (or that you redraw at 37.28). Areas at 37.28 m (543 m²) and 39.5 m (1932 m²) are YOUR survey values. Other yellow areas are still placeholders until you delineate those contours.</t>
+          <t>La cellule E de la ligne 37,28 m = volume d'eau total (m³) stocké dans le terrain lorsque la surface libre est à 37,28 m (en partant du radier vide). Les surfaces à 37,28 m (543 m²) et 39,5 m (1932 m²) sont VOS valeurs de levé. Les autres surfaces jaunes sont encore des placeholders jusqu'à ce que vous délimitez ces contours. Avec les placeholders actuels, V ≈ 558 m³ à 37,28 m ; ce volume changera si vous corrigez les surfaces intermédiaires.</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>V at boss stage (m³)</t>
+          <t>V au niveau patron (m³)</t>
         </is>
       </c>
       <c r="B26" s="19">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>← storage available when Qout = 2.4 m³/s (same WSE)</t>
+          <t>← volume disponible lorsque Qout = 2,4 m³/s (même NSE)</t>
         </is>
       </c>
     </row>

</xml_diff>